<commit_message>
Fix on minor issue architecture evalation
</commit_message>
<xml_diff>
--- a/outputs/evaluation/architecture/design/v1/CF_M01/CF_M01_arch_eval_avg.xlsx
+++ b/outputs/evaluation/architecture/design/v1/CF_M01/CF_M01_arch_eval_avg.xlsx
@@ -504,6 +504,8 @@
         <v>0.8611</v>
       </c>
     </row>
+    <row r="5"/>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -585,10 +587,8 @@
           <t>fixedType</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="B12" t="n">
+        <v>1</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>

</xml_diff>